<commit_message>
re-evaluation of req v1 and v2
</commit_message>
<xml_diff>
--- a/outputs/evaluation/requirement/design/v1/CF_M01/CF_M01_req_eval_avg.xlsx
+++ b/outputs/evaluation/requirement/design/v1/CF_M01/CF_M01_req_eval_avg.xlsx
@@ -624,10 +624,8 @@
           <t>fixes</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B22" t="n">
+        <v>0.4817</v>
       </c>
     </row>
   </sheetData>

</xml_diff>